<commit_message>
pac-man page layout clanup
</commit_message>
<xml_diff>
--- a/GD.codexalgorithm_contents_sheet.xlsx
+++ b/GD.codexalgorithm_contents_sheet.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="584" uniqueCount="142">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="584" uniqueCount="166">
   <si>
     <t>Timestamp</t>
   </si>
@@ -502,7 +502,7 @@
     <t>Is run locally, Runs on PC</t>
   </si>
   <si>
-    <t>Middle-earth: Shadow of Mordor (Nemesis System)</t>
+    <t>Middle-earth Shadow of Mordor (Nemesis System)</t>
   </si>
   <si>
     <t>racks player interactions with procedurally generated enemies.</t>
@@ -590,7 +590,7 @@
     <t>Is run on a server, Needs internet connection, Runs on PC, Runs on Playstation, Runs on Xbox</t>
   </si>
   <si>
-    <t>Bully AI (Grand Theft Auto: San Andreas)</t>
+    <t>Bully AI (Grand Theft Auto San Andreas)</t>
   </si>
   <si>
     <t>Rule-based system with an influence map to simulate pedestrian behavior. NPCs react based on the player's actions, creating emergent interactions such as fights, traffic accidents, and social dynamics.</t>
@@ -602,7 +602,7 @@
     <t>Used in controlling groups of animals (like birds or sheep), this AI uses Boids algorithm to simulate natural flocking behavior. The animals move together in groups with basic steering rules, like avoiding separation and maintaining cohesion.</t>
   </si>
   <si>
-    <t>Enemy AI (The Legend of Zelda: Ocarina of Time)</t>
+    <t>Enemy AI (The Legend of Zelda Ocarina of Time)</t>
   </si>
   <si>
     <t>State machine-based AI that handles enemy behavior, such as moving toward the player, attacking, or retreating. Each enemy has different states and transitions between them based on player interaction, health, and proximity.</t>
@@ -648,6 +648,78 @@
   </si>
   <si>
     <t>Real-time rendering</t>
+  </si>
+  <si>
+    <t>AI in alien isolation 2</t>
+  </si>
+  <si>
+    <t>AI of Forza drivers 2</t>
+  </si>
+  <si>
+    <t>No man's sky procedural generation 2</t>
+  </si>
+  <si>
+    <t>The Sims (Sim AI)2</t>
+  </si>
+  <si>
+    <t>Left 4 Dead (AI Director)2</t>
+  </si>
+  <si>
+    <t>Middle-earth Shadow of Mordor (Nemesis System)2</t>
+  </si>
+  <si>
+    <t>Halo (Combat AI)2</t>
+  </si>
+  <si>
+    <t>F.E.A.R. (Combat AI)2</t>
+  </si>
+  <si>
+    <t>Metal Gear Solid (Enemy AI)2</t>
+  </si>
+  <si>
+    <t>Chessmaster (Chess AI)2</t>
+  </si>
+  <si>
+    <t>Zerg Swarm AI (StarCraft)2</t>
+  </si>
+  <si>
+    <t>Giant Enemy Crab AI (Shenmue)2</t>
+  </si>
+  <si>
+    <t>The Predator AI (Alien vs. Predator)2</t>
+  </si>
+  <si>
+    <t>Civilization AI (Civilization series)2</t>
+  </si>
+  <si>
+    <t>Evolving AI Agents (Black &amp; White)2</t>
+  </si>
+  <si>
+    <t>Bully AI (Grand Theft Auto San Andreas)2</t>
+  </si>
+  <si>
+    <t>Flocking Behavior AI (Minecraft)2</t>
+  </si>
+  <si>
+    <t>Enemy AI (The Legend of Zelda Ocarina of Time)2</t>
+  </si>
+  <si>
+    <t>Goat AI (The Witcher 3)2</t>
+  </si>
+  <si>
+    <t>Evolving Enemy Behavior (Dead Rising)2</t>
+  </si>
+  <si>
+    <t>AI Companions (BioShock Infinite - Elizabeth)2</t>
+  </si>
+  <si>
+    <t>Dynamic Encounter AI (Dying Light)2</t>
+  </si>
+  <si>
+    <t>Autonomous Vehicle AI (Watch Dogs)2</t>
+  </si>
+  <si>
+    <t>Mind Control AI (Control)2</t>
   </si>
 </sst>
 </file>
@@ -2617,7 +2689,7 @@
         <v>45684.59649457176</v>
       </c>
       <c r="B33" s="17" t="s">
-        <v>61</v>
+        <v>142</v>
       </c>
       <c r="C33" s="17" t="s">
         <v>62</v>
@@ -2660,7 +2732,7 @@
         <v>45684.597505150465</v>
       </c>
       <c r="B34" s="14" t="s">
-        <v>69</v>
+        <v>143</v>
       </c>
       <c r="C34" s="14" t="s">
         <v>62</v>
@@ -2703,7 +2775,7 @@
         <v>45684.59914146991</v>
       </c>
       <c r="B35" s="17" t="s">
-        <v>73</v>
+        <v>144</v>
       </c>
       <c r="C35" s="17" t="s">
         <v>62</v>
@@ -2746,7 +2818,7 @@
         <v>45684.60510847223</v>
       </c>
       <c r="B36" s="14" t="s">
-        <v>80</v>
+        <v>145</v>
       </c>
       <c r="C36" s="14" t="s">
         <v>81</v>
@@ -2789,7 +2861,7 @@
         <v>45684.605959733795</v>
       </c>
       <c r="B37" s="17" t="s">
-        <v>86</v>
+        <v>146</v>
       </c>
       <c r="C37" s="17" t="s">
         <v>87</v>
@@ -2832,7 +2904,7 @@
         <v>45684.606631006944</v>
       </c>
       <c r="B38" s="14" t="s">
-        <v>93</v>
+        <v>147</v>
       </c>
       <c r="C38" s="14" t="s">
         <v>94</v>
@@ -2875,7 +2947,7 @@
         <v>45684.60733172453</v>
       </c>
       <c r="B39" s="17" t="s">
-        <v>95</v>
+        <v>148</v>
       </c>
       <c r="C39" s="17" t="s">
         <v>96</v>
@@ -2918,7 +2990,7 @@
         <v>45684.607788090274</v>
       </c>
       <c r="B40" s="14" t="s">
-        <v>98</v>
+        <v>149</v>
       </c>
       <c r="C40" s="14" t="s">
         <v>99</v>
@@ -2961,7 +3033,7 @@
         <v>45684.60839152778</v>
       </c>
       <c r="B41" s="17" t="s">
-        <v>100</v>
+        <v>150</v>
       </c>
       <c r="C41" s="17" t="s">
         <v>101</v>
@@ -3004,7 +3076,7 @@
         <v>45684.60918318287</v>
       </c>
       <c r="B42" s="14" t="s">
-        <v>103</v>
+        <v>151</v>
       </c>
       <c r="C42" s="14" t="s">
         <v>104</v>
@@ -3047,7 +3119,7 @@
         <v>45684.6122675</v>
       </c>
       <c r="B43" s="17" t="s">
-        <v>108</v>
+        <v>152</v>
       </c>
       <c r="C43" s="17" t="s">
         <v>109</v>
@@ -3090,7 +3162,7 @@
         <v>45684.61297810185</v>
       </c>
       <c r="B44" s="14" t="s">
-        <v>110</v>
+        <v>153</v>
       </c>
       <c r="C44" s="14" t="s">
         <v>111</v>
@@ -3133,7 +3205,7 @@
         <v>45684.61369174768</v>
       </c>
       <c r="B45" s="17" t="s">
-        <v>113</v>
+        <v>154</v>
       </c>
       <c r="C45" s="17" t="s">
         <v>114</v>
@@ -3176,7 +3248,7 @@
         <v>45684.614309745375</v>
       </c>
       <c r="B46" s="14" t="s">
-        <v>115</v>
+        <v>155</v>
       </c>
       <c r="C46" s="14" t="s">
         <v>116</v>
@@ -3219,7 +3291,7 @@
         <v>45684.615590925925</v>
       </c>
       <c r="B47" s="17" t="s">
-        <v>118</v>
+        <v>156</v>
       </c>
       <c r="C47" s="17" t="s">
         <v>119</v>
@@ -3262,7 +3334,7 @@
         <v>45684.61625390046</v>
       </c>
       <c r="B48" s="14" t="s">
-        <v>122</v>
+        <v>157</v>
       </c>
       <c r="C48" s="14" t="s">
         <v>123</v>
@@ -3305,7 +3377,7 @@
         <v>45684.617078587966</v>
       </c>
       <c r="B49" s="17" t="s">
-        <v>124</v>
+        <v>158</v>
       </c>
       <c r="C49" s="17" t="s">
         <v>125</v>
@@ -3348,7 +3420,7 @@
         <v>45684.617629988425</v>
       </c>
       <c r="B50" s="14" t="s">
-        <v>126</v>
+        <v>159</v>
       </c>
       <c r="C50" s="14" t="s">
         <v>127</v>
@@ -3391,7 +3463,7 @@
         <v>45684.61808251157</v>
       </c>
       <c r="B51" s="17" t="s">
-        <v>128</v>
+        <v>160</v>
       </c>
       <c r="C51" s="17" t="s">
         <v>129</v>
@@ -3434,7 +3506,7 @@
         <v>45684.618901168986</v>
       </c>
       <c r="B52" s="14" t="s">
-        <v>131</v>
+        <v>161</v>
       </c>
       <c r="C52" s="14" t="s">
         <v>132</v>
@@ -3477,7 +3549,7 @@
         <v>45684.61945407407</v>
       </c>
       <c r="B53" s="17" t="s">
-        <v>133</v>
+        <v>162</v>
       </c>
       <c r="C53" s="17" t="s">
         <v>134</v>
@@ -3520,7 +3592,7 @@
         <v>45684.61994938657</v>
       </c>
       <c r="B54" s="14" t="s">
-        <v>135</v>
+        <v>163</v>
       </c>
       <c r="C54" s="14" t="s">
         <v>136</v>
@@ -3563,7 +3635,7 @@
         <v>45684.62049341435</v>
       </c>
       <c r="B55" s="17" t="s">
-        <v>137</v>
+        <v>164</v>
       </c>
       <c r="C55" s="17" t="s">
         <v>138</v>
@@ -3606,7 +3678,7 @@
         <v>45684.62124706019</v>
       </c>
       <c r="B56" s="19" t="s">
-        <v>139</v>
+        <v>165</v>
       </c>
       <c r="C56" s="19" t="s">
         <v>140</v>

</xml_diff>